<commit_message>
Implement complete ETL pipeline orchestration and project documentation
</commit_message>
<xml_diff>
--- a/data/processed/cpi_processed.xlsx
+++ b/data/processed/cpi_processed.xlsx
@@ -472,7 +472,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -500,7 +500,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -528,7 +528,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -584,7 +584,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -612,7 +612,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -696,7 +696,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -724,7 +724,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -752,7 +752,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -780,7 +780,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -808,7 +808,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -836,7 +836,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -892,7 +892,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -920,7 +920,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -948,7 +948,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1004,7 +1004,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1032,7 +1032,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1060,7 +1060,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1088,7 +1088,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1116,7 +1116,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1144,7 +1144,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1172,7 +1172,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1200,7 +1200,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1256,7 +1256,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1284,7 +1284,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1312,7 +1312,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1340,7 +1340,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1396,7 +1396,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1424,7 +1424,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1452,7 +1452,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1480,7 +1480,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1508,7 +1508,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1536,7 +1536,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1564,7 +1564,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1592,7 +1592,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1620,7 +1620,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1648,7 +1648,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1676,7 +1676,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1704,7 +1704,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1732,7 +1732,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1760,7 +1760,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1788,7 +1788,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1816,7 +1816,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1844,7 +1844,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1872,7 +1872,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1900,7 +1900,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1928,7 +1928,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1956,7 +1956,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -1984,7 +1984,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2012,7 +2012,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2040,7 +2040,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2068,7 +2068,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2096,7 +2096,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2124,7 +2124,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2152,7 +2152,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2180,7 +2180,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2208,7 +2208,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2236,7 +2236,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2264,7 +2264,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2292,7 +2292,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2348,7 +2348,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2376,7 +2376,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2404,7 +2404,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2432,7 +2432,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2460,7 +2460,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2488,7 +2488,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2516,7 +2516,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2544,7 +2544,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2572,7 +2572,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2600,7 +2600,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2628,7 +2628,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2656,7 +2656,7 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2684,7 +2684,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2712,7 +2712,7 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2740,7 +2740,7 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2768,7 +2768,7 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2796,7 +2796,7 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2824,7 +2824,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2852,7 +2852,7 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2880,7 +2880,7 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2908,7 +2908,7 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2936,7 +2936,7 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2964,7 +2964,7 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -2992,7 +2992,7 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -3020,7 +3020,7 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -3048,7 +3048,7 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -3104,7 +3104,7 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -3132,7 +3132,7 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -3160,7 +3160,7 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -3188,7 +3188,7 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -3216,7 +3216,7 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -3244,7 +3244,7 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -3272,7 +3272,7 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -3300,7 +3300,7 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -3328,7 +3328,7 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -3356,7 +3356,7 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -3384,7 +3384,7 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -3412,7 +3412,7 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -3440,7 +3440,7 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -3468,7 +3468,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -3524,7 +3524,7 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -3552,7 +3552,7 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -3580,7 +3580,7 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -3608,7 +3608,7 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -3636,7 +3636,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -3664,7 +3664,7 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -3692,7 +3692,7 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -3720,7 +3720,7 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -3776,7 +3776,7 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -3804,7 +3804,7 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -3832,7 +3832,7 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -3860,7 +3860,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -3888,7 +3888,7 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -3916,7 +3916,7 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -3944,7 +3944,7 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -3972,7 +3972,7 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4000,7 +4000,7 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4028,7 +4028,7 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4056,7 +4056,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4084,7 +4084,7 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4112,7 +4112,7 @@
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4140,7 +4140,7 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4168,7 +4168,7 @@
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4196,7 +4196,7 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4224,7 +4224,7 @@
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4280,7 +4280,7 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4308,7 +4308,7 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4336,7 +4336,7 @@
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4364,7 +4364,7 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4392,7 +4392,7 @@
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4420,7 +4420,7 @@
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4448,7 +4448,7 @@
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4476,7 +4476,7 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4504,7 +4504,7 @@
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4532,7 +4532,7 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4560,7 +4560,7 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4616,7 +4616,7 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4644,7 +4644,7 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4672,7 +4672,7 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4700,7 +4700,7 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4728,7 +4728,7 @@
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4756,7 +4756,7 @@
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4784,7 +4784,7 @@
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4812,7 +4812,7 @@
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4840,7 +4840,7 @@
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4868,7 +4868,7 @@
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4896,7 +4896,7 @@
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4924,7 +4924,7 @@
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4952,7 +4952,7 @@
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -4980,7 +4980,7 @@
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5008,7 +5008,7 @@
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5036,7 +5036,7 @@
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5064,7 +5064,7 @@
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5092,7 +5092,7 @@
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5120,7 +5120,7 @@
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5148,7 +5148,7 @@
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5176,7 +5176,7 @@
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5204,7 +5204,7 @@
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5232,7 +5232,7 @@
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5260,7 +5260,7 @@
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5288,7 +5288,7 @@
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5316,7 +5316,7 @@
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5344,7 +5344,7 @@
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5372,7 +5372,7 @@
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5400,7 +5400,7 @@
       </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5428,7 +5428,7 @@
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5456,7 +5456,7 @@
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5484,7 +5484,7 @@
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5512,7 +5512,7 @@
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5540,7 +5540,7 @@
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5568,7 +5568,7 @@
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5596,7 +5596,7 @@
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5624,7 +5624,7 @@
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5652,7 +5652,7 @@
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5680,7 +5680,7 @@
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5708,7 +5708,7 @@
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5736,7 +5736,7 @@
       </c>
       <c r="F190" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5764,7 +5764,7 @@
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5792,7 +5792,7 @@
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5820,7 +5820,7 @@
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5848,7 +5848,7 @@
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5876,7 +5876,7 @@
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5904,7 +5904,7 @@
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5932,7 +5932,7 @@
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5960,7 +5960,7 @@
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -5988,7 +5988,7 @@
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6016,7 +6016,7 @@
       </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6044,7 +6044,7 @@
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6072,7 +6072,7 @@
       </c>
       <c r="F202" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6100,7 +6100,7 @@
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6128,7 +6128,7 @@
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6156,7 +6156,7 @@
       </c>
       <c r="F205" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6184,7 +6184,7 @@
       </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6212,7 +6212,7 @@
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6240,7 +6240,7 @@
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6268,7 +6268,7 @@
       </c>
       <c r="F209" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6296,7 +6296,7 @@
       </c>
       <c r="F210" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6324,7 +6324,7 @@
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6352,7 +6352,7 @@
       </c>
       <c r="F212" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6380,7 +6380,7 @@
       </c>
       <c r="F213" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6408,7 +6408,7 @@
       </c>
       <c r="F214" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6436,7 +6436,7 @@
       </c>
       <c r="F215" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6464,7 +6464,7 @@
       </c>
       <c r="F216" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6492,7 +6492,7 @@
       </c>
       <c r="F217" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6520,7 +6520,7 @@
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6548,7 +6548,7 @@
       </c>
       <c r="F219" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6576,7 +6576,7 @@
       </c>
       <c r="F220" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6604,7 +6604,7 @@
       </c>
       <c r="F221" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6632,7 +6632,7 @@
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6660,7 +6660,7 @@
       </c>
       <c r="F223" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6688,7 +6688,7 @@
       </c>
       <c r="F224" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6716,7 +6716,7 @@
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6744,7 +6744,7 @@
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6772,7 +6772,7 @@
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6800,7 +6800,7 @@
       </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6828,7 +6828,7 @@
       </c>
       <c r="F229" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6856,7 +6856,7 @@
       </c>
       <c r="F230" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6884,7 +6884,7 @@
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6912,7 +6912,7 @@
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6940,7 +6940,7 @@
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6968,7 +6968,7 @@
       </c>
       <c r="F234" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -6996,7 +6996,7 @@
       </c>
       <c r="F235" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -7024,7 +7024,7 @@
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -7052,7 +7052,7 @@
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -7080,7 +7080,7 @@
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -7108,7 +7108,7 @@
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -7136,7 +7136,7 @@
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -7164,7 +7164,7 @@
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -7192,7 +7192,7 @@
       </c>
       <c r="F242" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -7220,7 +7220,7 @@
       </c>
       <c r="F243" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -7248,7 +7248,7 @@
       </c>
       <c r="F244" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -7276,7 +7276,7 @@
       </c>
       <c r="F245" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -7304,7 +7304,7 @@
       </c>
       <c r="F246" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -7332,7 +7332,7 @@
       </c>
       <c r="F247" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -7360,7 +7360,7 @@
       </c>
       <c r="F248" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -7388,7 +7388,7 @@
       </c>
       <c r="F249" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -7416,7 +7416,7 @@
       </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -7444,7 +7444,7 @@
       </c>
       <c r="F251" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -7472,7 +7472,7 @@
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -7500,7 +7500,7 @@
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -7528,7 +7528,7 @@
       </c>
       <c r="F254" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -7556,7 +7556,7 @@
       </c>
       <c r="F255" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -7584,7 +7584,7 @@
       </c>
       <c r="F256" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -7612,7 +7612,7 @@
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -7640,7 +7640,7 @@
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -7668,7 +7668,7 @@
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -7696,7 +7696,7 @@
       </c>
       <c r="F260" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -7724,7 +7724,7 @@
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -7752,7 +7752,7 @@
       </c>
       <c r="F262" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -7780,7 +7780,7 @@
       </c>
       <c r="F263" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -7808,7 +7808,7 @@
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -7836,7 +7836,7 @@
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -7864,7 +7864,7 @@
       </c>
       <c r="F266" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -7892,7 +7892,7 @@
       </c>
       <c r="F267" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -7920,7 +7920,7 @@
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -7948,7 +7948,7 @@
       </c>
       <c r="F269" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -7976,7 +7976,7 @@
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -8004,7 +8004,7 @@
       </c>
       <c r="F271" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -8030,7 +8030,7 @@
       </c>
       <c r="F272" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -8056,7 +8056,7 @@
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -8082,7 +8082,7 @@
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -8108,7 +8108,7 @@
       </c>
       <c r="F275" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -8134,7 +8134,7 @@
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -8160,7 +8160,7 @@
       </c>
       <c r="F277" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -8186,7 +8186,7 @@
       </c>
       <c r="F278" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -8212,7 +8212,7 @@
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -8238,7 +8238,7 @@
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -8264,7 +8264,7 @@
       </c>
       <c r="F281" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -8290,7 +8290,7 @@
       </c>
       <c r="F282" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -8316,7 +8316,7 @@
       </c>
       <c r="F283" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -8342,7 +8342,7 @@
       </c>
       <c r="F284" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -8368,7 +8368,7 @@
       </c>
       <c r="F285" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -8394,7 +8394,7 @@
       </c>
       <c r="F286" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -8420,7 +8420,7 @@
       </c>
       <c r="F287" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -8446,7 +8446,7 @@
       </c>
       <c r="F288" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -8472,7 +8472,7 @@
       </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -8498,7 +8498,7 @@
       </c>
       <c r="F290" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -8524,7 +8524,7 @@
       </c>
       <c r="F291" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -8550,7 +8550,7 @@
       </c>
       <c r="F292" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -8576,7 +8576,7 @@
       </c>
       <c r="F293" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -8602,7 +8602,7 @@
       </c>
       <c r="F294" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -8628,7 +8628,7 @@
       </c>
       <c r="F295" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -8654,7 +8654,7 @@
       </c>
       <c r="F296" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -8680,7 +8680,7 @@
       </c>
       <c r="F297" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -8706,7 +8706,7 @@
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -8732,7 +8732,7 @@
       </c>
       <c r="F299" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -8758,7 +8758,7 @@
       </c>
       <c r="F300" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>
@@ -8784,7 +8784,7 @@
       </c>
       <c r="F301" t="inlineStr">
         <is>
-          <t>2026-07-28 01:30:01</t>
+          <t>2026-07-28 08:51:22</t>
         </is>
       </c>
     </row>

</xml_diff>